<commit_message>
sync updated run-of-show and add 展旗 gallery image
</commit_message>
<xml_diff>
--- a/assets/天狮2026非洲区表彰大会_官方执行总流程表.xlsx
+++ b/assets/天狮2026非洲区表彰大会_官方执行总流程表.xlsx
@@ -11,7 +11,7 @@
     <sheet name="分公司参会人数" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Run of Show'!$A$9:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Run of Show'!$A$9:$H$39</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="174">
   <si>
     <t>天狮 2026 非洲区表彰大会（TIENS 2026 Africa Regional Recognition Convention）</t>
   </si>
@@ -93,7 +93,7 @@
     <t>16:00 - 18:00  |  预热篇章：万人集结与狂欢热场  |  核心任务：完成万人入场安检，拉升现场温度，完成开场前全链路确认</t>
   </si>
   <si>
-    <t>16:00 - 17:30</t>
+    <t>16:00 - 17:20</t>
   </si>
   <si>
     <t>预热篇章</t>
@@ -102,31 +102,46 @@
     <t>万人入场 &amp; 区域拉歌</t>
   </si>
   <si>
-    <t>万人有序入场与安检，按国家方阵落位。</t>
-  </si>
-  <si>
-    <t>大屏循环天狮全球宣传片；主持人引导拉歌互动。</t>
-  </si>
-  <si>
-    <t>大屏循环宣传片；安保广播引导。</t>
-  </si>
-  <si>
-    <t>17:30 - 17:45</t>
+    <t>万人有序入场与安检，快速完成分区落位。</t>
+  </si>
+  <si>
+    <t>非洲各国代表团及本地经销商按区块入场；大屏循环宣传片，主持人引导分区拉歌。</t>
+  </si>
+  <si>
+    <t>入场进行曲+分区互动麦克；安保广播引导。</t>
+  </si>
+  <si>
+    <t>17:20 - 17:32</t>
   </si>
   <si>
     <t>热场高潮：天狮专属舞蹈秀</t>
   </si>
   <si>
-    <t>舞蹈团队高能热场，形成首轮情绪峰值。</t>
-  </si>
-  <si>
-    <t>本地专业伴舞团队领舞，全场万人共舞。</t>
+    <t>完成开场前第一轮情绪点火。</t>
+  </si>
+  <si>
+    <t>本地专业伴舞团队领舞，带动全场共舞。</t>
   </si>
   <si>
     <t>动感BGM+追光+舞台全彩灯。</t>
   </si>
   <si>
-    <t>17:45 - 18:00</t>
+    <t>17:32 - 17:48</t>
+  </si>
+  <si>
+    <t>非洲各国方阵举旗入场</t>
+  </si>
+  <si>
+    <t>强化国际阵容展示与仪式感。</t>
+  </si>
+  <si>
+    <t>各非洲国家方阵代表手举本国国旗入场，按“后场→前场”路线绕场一圈后落位；随后进入分区拉歌互动。</t>
+  </si>
+  <si>
+    <t>国家方阵播报+国旗特写；动线安保分段控场。</t>
+  </si>
+  <si>
+    <t>17:48 - 18:00</t>
   </si>
   <si>
     <t>VIP莅临 &amp; 倒计时准备</t>
@@ -135,16 +150,16 @@
     <t>确保VIP准时入座并完成开场倒计时准备。</t>
   </si>
   <si>
-    <t>17:59全场主灯变暗，大屏开启60秒倒计时。</t>
-  </si>
-  <si>
-    <t>倒计时视频+低频鼓点渐强。</t>
+    <t>政府官员、总部领导及非洲区高管在礼宾及安保引导下入座；17:59开启60秒倒计时。</t>
+  </si>
+  <si>
+    <t>主灯渐暗；倒计时视频+低频鼓点。</t>
   </si>
   <si>
     <t>18:00 - 18:45  |  第一篇章：盛典启幕与领袖愿景  |  核心任务：准点开场，建立国家级礼仪感与政商共赢格局</t>
   </si>
   <si>
-    <t>18:00 - 18:10</t>
+    <t>18:00 - 18:08</t>
   </si>
   <si>
     <t>第一篇章</t>
@@ -162,7 +177,7 @@
     <t>主扩全开；国旗与司歌画面切换。</t>
   </si>
   <si>
-    <t>18:10 - 18:15</t>
+    <t>18:08 - 18:13</t>
   </si>
   <si>
     <t>东道主致欢迎词</t>
@@ -177,7 +192,7 @@
     <t>讲台麦启用；欢迎词主题板上屏。</t>
   </si>
   <si>
-    <t>18:15 - 18:25</t>
+    <t>18:13 - 18:23</t>
   </si>
   <si>
     <t>董事局主席致辞（视频）</t>
@@ -192,7 +207,7 @@
     <t>视频服务器A/B备份；字幕核对。</t>
   </si>
   <si>
-    <t>18:25 - 18:35</t>
+    <t>18:23 - 18:33</t>
   </si>
   <si>
     <t>高级经销商代表致辞</t>
@@ -207,7 +222,7 @@
     <t>追光锁定；观众反应镜头实时上屏。</t>
   </si>
   <si>
-    <t>18:35 - 18:45</t>
+    <t>18:33 - 18:45</t>
   </si>
   <si>
     <t>多哥政府官员致辞</t>
@@ -243,7 +258,7 @@
     <t>8星视觉特效；名单滚动；颁奖音乐。</t>
   </si>
   <si>
-    <t>18:50 - 18:58</t>
+    <t>18:50 - 19:00</t>
   </si>
   <si>
     <t>天狮产品走秀</t>
@@ -258,7 +273,7 @@
     <t>时尚BGM；灯光追踪；产品特写。</t>
   </si>
   <si>
-    <t>18:58 - 19:07</t>
+    <t>19:00 - 19:09</t>
   </si>
   <si>
     <t>新晋铜狮颁奖</t>
@@ -273,7 +288,7 @@
     <t>铜狮立体特效；动线引导。</t>
   </si>
   <si>
-    <t>19:07 - 19:13</t>
+    <t>19:09 - 19:15</t>
   </si>
   <si>
     <t>新晋银狮颁奖</t>
@@ -288,7 +303,7 @@
     <t>银狮特效；名单滚动。</t>
   </si>
   <si>
-    <t>19:13 - 19:20</t>
+    <t>19:15 - 19:20</t>
   </si>
   <si>
     <t>新晋金狮颁奖</t>
@@ -306,7 +321,7 @@
     <t>19:20 - 19:40  |  第三篇章：东方力量与狮军出征  |  核心任务：以文化冲击承接情绪，导入战斗团队授勋</t>
   </si>
   <si>
-    <t>19:20 - 19:30</t>
+    <t>19:20 - 19:29</t>
   </si>
   <si>
     <t>第三篇章</t>
@@ -324,7 +339,7 @@
     <t>鼓点与灯光节奏同步。</t>
   </si>
   <si>
-    <t>19:30 - 19:40</t>
+    <t>19:29 - 19:36</t>
   </si>
   <si>
     <t>狮军授勋（Armée des Lions）</t>
@@ -339,10 +354,25 @@
     <t>授勋名单核对；道具提前分组。</t>
   </si>
   <si>
+    <t>19:36 - 19:40</t>
+  </si>
+  <si>
+    <t>双旗接力展开仪式</t>
+  </si>
+  <si>
+    <t>通过高规格旗阵仪式强化团队精神与领袖象征。</t>
+  </si>
+  <si>
+    <t>两面20米长旗子分别接力展开：一面狮旗（前场→后场），一面董事长画像旗（后场→前场）。</t>
+  </si>
+  <si>
+    <t>双旗同时起旗；主追光分左右两路；航拍/摇臂抓全景。</t>
+  </si>
+  <si>
     <t>19:40 - 20:30  |  第四篇章：极速引擎、狂欢派对与巅峰财富  |  核心任务：演艺狂欢与硬件大奖交替轰炸，打造绝对情绪核爆点</t>
   </si>
   <si>
-    <t>19:40 - 19:55</t>
+    <t>19:40 - 19:54</t>
   </si>
   <si>
     <t>第四篇章</t>
@@ -360,7 +390,7 @@
     <t>低频引擎音效；机车灯控联动。</t>
   </si>
   <si>
-    <t>19:55 - 20:05</t>
+    <t>19:54 - 20:06</t>
   </si>
   <si>
     <t>多哥本土重磅演艺狂欢</t>
@@ -375,7 +405,7 @@
     <t>艺人进退场计时；舞台安全员前置。</t>
   </si>
   <si>
-    <t>20:05 - 20:15</t>
+    <t>20:06 - 20:17</t>
   </si>
   <si>
     <t>豪华汽车大奖（Prix Voiture）</t>
@@ -390,7 +420,7 @@
     <t>豪车视觉包；礼仪道具到位。</t>
   </si>
   <si>
-    <t>20:15 - 20:30</t>
+    <t>20:17 - 20:30</t>
   </si>
   <si>
     <t>豪华别墅大奖（Prix Villa）</t>
@@ -408,7 +438,7 @@
     <t>20:30 - 20:55  |  第五篇章：统帅出征与圆满落幕  |  核心任务：把现场热度转化为下半年市场战斗力</t>
   </si>
   <si>
-    <t>20:30 - 20:45</t>
+    <t>20:30 - 20:43</t>
   </si>
   <si>
     <t>第五篇章</t>
@@ -426,7 +456,7 @@
     <t>总裁上场音乐；政策要点上屏。</t>
   </si>
   <si>
-    <t>20:45 - 20:50</t>
+    <t>20:43 - 20:49</t>
   </si>
   <si>
     <t>压轴大合影</t>
@@ -441,7 +471,7 @@
     <t>摄影机位预排；站位图执行。</t>
   </si>
   <si>
-    <t>20:50 - 20:55</t>
+    <t>20:49 - 20:55</t>
   </si>
   <si>
     <t>欢送与退场</t>
@@ -454,6 +484,9 @@
   </si>
   <si>
     <t>退场广播循环；外场探照灯开启。</t>
+  </si>
+  <si>
+    <t>备注：本表为总控执行版，建议会前D-3完成全流程彩排；D-1完成音视频、灯光、礼宾、安保四线联排。</t>
   </si>
   <si>
     <t>各分公司参加经销商人员（预计）</t>
@@ -1009,7 +1042,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -1021,6 +1054,30 @@
       <left style="thin">
         <color rgb="FFD9D9D9"/>
       </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="FFD9D9D9"/>
       </right>
@@ -1193,7 +1250,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
@@ -1205,34 +1262,34 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="10">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="12">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="13">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="14">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="16" borderId="0">
@@ -1317,7 +1374,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1328,27 +1385,20 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1358,34 +1408,34 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1737,7 +1787,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1751,758 +1801,812 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:8">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:8">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="16" t="s">
+      <c r="B4" s="14"/>
+      <c r="C4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="15"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="14"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:8">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="16" t="s">
+      <c r="B5" s="14"/>
+      <c r="C5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="15"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="14"/>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:8">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="14"/>
+      <c r="C6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="15"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="14"/>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:8">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="15"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="14"/>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="18" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:8">
-      <c r="A10" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="21" t="s">
+      <c r="A10" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="15"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="14"/>
     </row>
     <row r="11" ht="56" customHeight="1" spans="1:8">
-      <c r="A11" s="22">
+      <c r="A11" s="21">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="G11" s="23" t="s">
+      <c r="G11" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="H11" s="23" t="s">
+      <c r="H11" s="22" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" ht="56" customHeight="1" spans="1:8">
-      <c r="A12" s="24">
+      <c r="A12" s="23">
         <v>2</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F12" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="24" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" ht="56" customHeight="1" spans="1:8">
-      <c r="A13" s="22">
+      <c r="A13" s="21">
         <v>3</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H13" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1" spans="1:8">
-      <c r="A14" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="21" t="s">
+      <c r="H13" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1" spans="1:8">
+      <c r="A14" s="23">
+        <v>4</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="15"/>
-    </row>
-    <row r="15" ht="56" customHeight="1" spans="1:8">
-      <c r="A15" s="24">
-        <v>4</v>
-      </c>
-      <c r="B15" s="24" t="s">
+      <c r="C14" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="E14" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="F14" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="G14" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="H14" s="24" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1" spans="1:8">
+      <c r="A15" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="14"/>
+    </row>
+    <row r="16" ht="56" customHeight="1" spans="1:8">
+      <c r="A16" s="21">
+        <v>5</v>
+      </c>
+      <c r="B16" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="H15" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" ht="56" customHeight="1" spans="1:8">
-      <c r="A16" s="22">
-        <v>5</v>
-      </c>
-      <c r="B16" s="22" t="s">
+      <c r="C16" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="F16" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="23" t="s">
+      <c r="G16" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="H16" s="23" t="s">
+      <c r="H16" s="22" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" ht="56" customHeight="1" spans="1:8">
-      <c r="A17" s="24">
+      <c r="A17" s="23">
         <v>6</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="25" t="s">
+      <c r="C17" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="E17" s="25" t="s">
+      <c r="E17" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="F17" s="25" t="s">
+      <c r="F17" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="25" t="s">
+      <c r="G17" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="H17" s="25" t="s">
+      <c r="H17" s="24" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="18" ht="56" customHeight="1" spans="1:8">
-      <c r="A18" s="22">
+      <c r="A18" s="21">
         <v>7</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18" s="23" t="s">
+      <c r="C18" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="F18" s="23" t="s">
+      <c r="F18" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="G18" s="23" t="s">
+      <c r="G18" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="H18" s="23" t="s">
+      <c r="H18" s="22" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="19" ht="56" customHeight="1" spans="1:8">
-      <c r="A19" s="24">
+      <c r="A19" s="23">
         <v>8</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="C19" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" s="25" t="s">
+      <c r="C19" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E19" s="25" t="s">
+      <c r="E19" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="25" t="s">
+      <c r="F19" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G19" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="H19" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:8">
-      <c r="A20" s="20" t="s">
-        <v>18</v>
+      <c r="H19" s="24" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" ht="56" customHeight="1" spans="1:8">
+      <c r="A20" s="21">
+        <v>9</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="15"/>
-    </row>
-    <row r="21" ht="56" customHeight="1" spans="1:8">
-      <c r="A21" s="22">
-        <v>9</v>
-      </c>
-      <c r="B21" s="22" t="s">
+      <c r="C20" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="E20" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="F20" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="G20" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="23" t="s">
+      <c r="H20" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1" spans="1:8">
+      <c r="A21" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="G21" s="23" t="s">
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="14"/>
+    </row>
+    <row r="22" ht="56" customHeight="1" spans="1:8">
+      <c r="A22" s="23">
+        <v>10</v>
+      </c>
+      <c r="B22" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="H21" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" ht="56" customHeight="1" spans="1:8">
-      <c r="A22" s="24">
-        <v>10</v>
-      </c>
-      <c r="B22" s="24" t="s">
+      <c r="C22" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="E22" s="25" t="s">
+      <c r="E22" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="F22" s="25" t="s">
+      <c r="F22" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="G22" s="25" t="s">
+      <c r="G22" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="H22" s="25" t="s">
+      <c r="H22" s="24" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="23" ht="56" customHeight="1" spans="1:8">
-      <c r="A23" s="22">
+      <c r="A23" s="21">
         <v>11</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" s="23" t="s">
+      <c r="C23" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="E23" s="23" t="s">
+      <c r="E23" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="G23" s="23" t="s">
+      <c r="G23" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="22" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="24" ht="56" customHeight="1" spans="1:8">
-      <c r="A24" s="24">
+      <c r="A24" s="23">
         <v>12</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="C24" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" s="25" t="s">
+      <c r="C24" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="E24" s="25" t="s">
+      <c r="E24" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="F24" s="25" t="s">
+      <c r="F24" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="G24" s="25" t="s">
+      <c r="G24" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="H24" s="25" t="s">
+      <c r="H24" s="24" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="25" ht="56" customHeight="1" spans="1:8">
-      <c r="A25" s="22">
+      <c r="A25" s="21">
         <v>13</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="C25" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D25" s="23" t="s">
+      <c r="C25" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D25" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="E25" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="F25" s="23" t="s">
+      <c r="F25" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="G25" s="23" t="s">
+      <c r="G25" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="H25" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1" spans="1:8">
-      <c r="A26" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B26" s="21" t="s">
+      <c r="H25" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" ht="56" customHeight="1" spans="1:8">
+      <c r="A26" s="23">
+        <v>14</v>
+      </c>
+      <c r="B26" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="15"/>
-    </row>
-    <row r="27" ht="56" customHeight="1" spans="1:8">
-      <c r="A27" s="24">
-        <v>14</v>
-      </c>
-      <c r="B27" s="24" t="s">
+      <c r="C26" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="D26" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="C27" s="25" t="s">
+      <c r="E26" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="25" t="s">
+      <c r="F26" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="E27" s="25" t="s">
+      <c r="G26" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="F27" s="25" t="s">
+      <c r="H26" s="24" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1" spans="1:8">
+      <c r="A27" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="G27" s="25" t="s">
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="14"/>
+    </row>
+    <row r="28" ht="56" customHeight="1" spans="1:8">
+      <c r="A28" s="21">
+        <v>15</v>
+      </c>
+      <c r="B28" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="H27" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28" ht="56" customHeight="1" spans="1:8">
-      <c r="A28" s="22">
-        <v>15</v>
-      </c>
-      <c r="B28" s="22" t="s">
+      <c r="C28" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="C28" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="F28" s="23" t="s">
+      <c r="F28" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="G28" s="23" t="s">
+      <c r="G28" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="H28" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1" spans="1:8">
-      <c r="A29" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="21" t="s">
+      <c r="H28" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" ht="56" customHeight="1" spans="1:8">
+      <c r="A29" s="23">
+        <v>16</v>
+      </c>
+      <c r="B29" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="15"/>
+      <c r="C29" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="D29" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="E29" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="F29" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="G29" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="30" ht="56" customHeight="1" spans="1:8">
-      <c r="A30" s="24">
-        <v>16</v>
-      </c>
-      <c r="B30" s="24" t="s">
-        <v>103</v>
-      </c>
-      <c r="C30" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="D30" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="E30" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="F30" s="25" t="s">
+      <c r="A30" s="21">
+        <v>17</v>
+      </c>
+      <c r="B30" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="G30" s="25" t="s">
+      <c r="C30" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="D30" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="H30" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="31" ht="56" customHeight="1" spans="1:8">
-      <c r="A31" s="22">
-        <v>17</v>
-      </c>
-      <c r="B31" s="22" t="s">
+      <c r="E30" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="C31" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="D31" s="23" t="s">
+      <c r="F30" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="G30" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="H30" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1" spans="1:8">
+      <c r="A31" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="G31" s="23" t="s">
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="14"/>
+    </row>
+    <row r="32" ht="56" customHeight="1" spans="1:8">
+      <c r="A32" s="23">
+        <v>18</v>
+      </c>
+      <c r="B32" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="H31" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="32" ht="56" customHeight="1" spans="1:8">
-      <c r="A32" s="24">
-        <v>18</v>
-      </c>
-      <c r="B32" s="24" t="s">
+      <c r="C32" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="C32" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="D32" s="25" t="s">
+      <c r="D32" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="E32" s="25" t="s">
+      <c r="E32" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="F32" s="25" t="s">
+      <c r="F32" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="G32" s="25" t="s">
+      <c r="G32" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="H32" s="25" t="s">
+      <c r="H32" s="24" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="33" ht="56" customHeight="1" spans="1:8">
-      <c r="A33" s="22">
+      <c r="A33" s="21">
         <v>19</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="C33" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="D33" s="23" t="s">
+      <c r="C33" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="E33" s="23" t="s">
+      <c r="E33" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="F33" s="23" t="s">
+      <c r="F33" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="G33" s="23" t="s">
+      <c r="G33" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="H33" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1" spans="1:8">
-      <c r="A34" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" s="21" t="s">
+      <c r="H33" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" ht="56" customHeight="1" spans="1:8">
+      <c r="A34" s="23">
+        <v>20</v>
+      </c>
+      <c r="B34" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="15"/>
+      <c r="C34" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="F34" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="G34" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="H34" s="24" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="35" ht="56" customHeight="1" spans="1:8">
-      <c r="A35" s="24">
-        <v>20</v>
-      </c>
-      <c r="B35" s="24" t="s">
-        <v>125</v>
-      </c>
-      <c r="C35" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="D35" s="25" t="s">
-        <v>127</v>
-      </c>
-      <c r="E35" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="F35" s="25" t="s">
+      <c r="A35" s="21">
+        <v>21</v>
+      </c>
+      <c r="B35" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="G35" s="25" t="s">
+      <c r="C35" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D35" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H35" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="36" ht="56" customHeight="1" spans="1:8">
-      <c r="A36" s="22">
-        <v>21</v>
-      </c>
-      <c r="B36" s="22" t="s">
+      <c r="E35" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="C36" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="D36" s="23" t="s">
+      <c r="F35" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="E36" s="23" t="s">
+      <c r="G35" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="F36" s="23" t="s">
+      <c r="H35" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1" spans="1:8">
+      <c r="A36" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="G36" s="23" t="s">
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="14"/>
+    </row>
+    <row r="37" ht="56" customHeight="1" spans="1:8">
+      <c r="A37" s="23">
+        <v>22</v>
+      </c>
+      <c r="B37" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="H36" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="37" ht="56" customHeight="1" spans="1:8">
-      <c r="A37" s="24">
-        <v>22</v>
-      </c>
-      <c r="B37" s="24" t="s">
+      <c r="C37" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="C37" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="D37" s="25" t="s">
+      <c r="D37" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="E37" s="25" t="s">
+      <c r="E37" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="F37" s="25" t="s">
+      <c r="F37" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="G37" s="25" t="s">
+      <c r="G37" s="24" t="s">
         <v>140</v>
       </c>
-      <c r="H37" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" ht="14.5" customHeight="1" spans="1:8">
-      <c r="A39" s="26"/>
+      <c r="H37" s="24" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" ht="56" customHeight="1" spans="1:8">
+      <c r="A38" s="21">
+        <v>23</v>
+      </c>
+      <c r="B38" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="F38" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="G38" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="H38" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="39" ht="56" customHeight="1" spans="1:8">
+      <c r="A39" s="23">
+        <v>24</v>
+      </c>
+      <c r="B39" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="C39" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="D39" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="E39" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="F39" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="G39" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="H39" s="24" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41" ht="14.5" customHeight="1" spans="1:8">
+      <c r="A41" s="25" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A9:H37" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A9:H39" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <mergeCells count="17">
@@ -2517,12 +2621,12 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="A41:H41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2544,185 +2648,185 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:6">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" spans="1:6">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:6">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" spans="1:6">
       <c r="A4" s="3">
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="D4" s="4">
+        <v>159</v>
+      </c>
+      <c r="D4" s="3">
         <v>500</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>1000</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:6">
-      <c r="A5" s="6">
+      <c r="F4" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" spans="1:6">
+      <c r="A5" s="5">
         <v>2</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="D5" s="7">
+      <c r="B5" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5" s="5">
         <v>50</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="5">
         <v>50</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:6">
+      <c r="F5" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" spans="1:6">
       <c r="A6" s="3">
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D6" s="4">
+        <v>164</v>
+      </c>
+      <c r="D6" s="3">
         <v>20</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>20</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:6">
-      <c r="A7" s="6">
+      <c r="F6" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" spans="1:6">
+      <c r="A7" s="5">
         <v>4</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="D7" s="7">
+      <c r="B7" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="D7" s="5">
         <v>50</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="5">
         <v>100</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:6">
+      <c r="F7" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" spans="1:6">
       <c r="A8" s="3">
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="D8" s="4">
+        <v>168</v>
+      </c>
+      <c r="D8" s="3">
         <v>5</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>10</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:6">
-      <c r="A9" s="6">
+      <c r="F8" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" spans="1:6">
+      <c r="A9" s="5">
         <v>6</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="D9" s="7">
+      <c r="B9" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="5">
         <v>20</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="5">
         <v>50</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:6">
+      <c r="F9" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" spans="1:6">
       <c r="A10" s="3">
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="D10" s="4">
+        <v>168</v>
+      </c>
+      <c r="D10" s="3">
         <v>5</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>10</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" ht="16.5" spans="1:6">
-      <c r="A11" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="B11" s="9"/>
+      <c r="F10" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" spans="1:6">
+      <c r="A11" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11" s="8"/>
       <c r="C11" s="9"/>
-      <c r="D11" s="10">
+      <c r="D11" s="7">
         <f>SUM(D4:D10)</f>
         <v>650</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="7">
         <f>SUM(E4:E10)</f>
         <v>1240</v>
       </c>
-      <c r="F11" s="11" t="s">
-        <v>162</v>
+      <c r="F11" s="10" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>